<commit_message>
Exercise 6, need to check it and clean the code
</commit_message>
<xml_diff>
--- a/Problem 5/TF_Parameters.xlsx
+++ b/Problem 5/TF_Parameters.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="8960" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="10233" uniqueCount="47">
   <si>
     <t>TransferFunction</t>
   </si>
@@ -535,16 +535,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1DCA3DE-9CFE-4C27-815C-DA57E594799D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1DCA3DE-9CFE-4C27-815C-DA57E594799D}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="2" width="15.21875" customWidth="1"/>
-    <col min="3" max="3" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="14.77734375" customWidth="true"/>
+    <col min="2" max="2" width="15.21875" customWidth="true"/>
+    <col min="3" max="3" width="11.5546875" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -555,7 +555,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -566,7 +566,7 @@
         <v>128.3987000997212</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -577,7 +577,7 @@
         <v>205.47293943459476</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -588,7 +588,7 @@
         <v>233.53955069205435</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -599,7 +599,7 @@
         <v>144.15927494199957</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -610,7 +610,7 @@
         <v>23.692593188913669</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -621,7 +621,7 @@
         <v>81.1160396871431</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -632,7 +632,7 @@
         <v>89.395584681261596</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -649,16 +649,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A0EAC4A-EE48-4914-A0C3-87ADA4F1E9F0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A0EAC4A-EE48-4914-A0C3-87ADA4F1E9F0}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="2" width="14.5546875" customWidth="1"/>
-    <col min="3" max="3" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="14.77734375" customWidth="true"/>
+    <col min="2" max="2" width="14.5546875" customWidth="true"/>
+    <col min="3" max="3" width="11.5546875" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -669,7 +669,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -680,7 +680,7 @@
         <v>174.76359658211501</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -691,7 +691,7 @@
         <v>279.51478537738473</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -702,7 +702,7 @@
         <v>306.35003683037371</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -713,7 +713,7 @@
         <v>133.74355924842379</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -724,7 +724,7 @@
         <v>123.22645885432243</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -735,7 +735,7 @@
         <v>90.697912922583697</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -746,7 +746,7 @@
         <v>46.546443659500454</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -767,10 +767,10 @@
   <dimension ref="A1:D13"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.77734375" customWidth="true"/>
-    <col min="2" max="2" width="14.77734375" customWidth="true"/>
-    <col min="3" max="3" width="13.5546875" customWidth="true"/>
-    <col min="4" max="4" width="13.77734375" customWidth="true"/>
+    <col min="1" max="1" width="8.86328125" customWidth="true"/>
+    <col min="2" max="2" width="14.59765625" customWidth="true"/>
+    <col min="3" max="3" width="13.796875" customWidth="true"/>
+    <col min="4" max="4" width="13.6640625" customWidth="true"/>
   </cols>
   <sheetData>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
@@ -840,7 +840,7 @@
         <v>0.23927080437932036</v>
       </c>
       <c r="D5" s="0">
-        <v>129.93522414268981</v>
+        <v>129.9352241426898</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
@@ -896,7 +896,7 @@
         <v>0.23927080437932036</v>
       </c>
       <c r="D9" s="0">
-        <v>129.93522414268981</v>
+        <v>129.9352241426898</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
@@ -952,7 +952,7 @@
         <v>0.23927080437932036</v>
       </c>
       <c r="D13" s="0">
-        <v>129.93522414268981</v>
+        <v>129.9352241426898</v>
       </c>
     </row>
   </sheetData>
@@ -965,21 +965,21 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" customWidth="true"/>
-    <col min="2" max="2" width="13.88671875" customWidth="true"/>
-    <col min="3" max="3" width="15" customWidth="true"/>
-    <col min="4" max="4" width="25.21875" customWidth="true"/>
-    <col min="5" max="5" width="26.33203125" customWidth="true"/>
-    <col min="6" max="6" width="20.5546875" customWidth="true"/>
-    <col min="7" max="7" width="34.33203125" customWidth="true"/>
-    <col min="8" max="8" width="21.6640625" customWidth="true"/>
-    <col min="9" max="9" width="33.6640625" customWidth="true"/>
-    <col min="10" max="10" width="22.77734375" customWidth="true"/>
-    <col min="11" max="11" width="23.88671875" customWidth="true"/>
-    <col min="12" max="12" width="18.109375" customWidth="true"/>
-    <col min="13" max="13" width="31.88671875" customWidth="true"/>
-    <col min="14" max="14" width="19.21875" customWidth="true"/>
-    <col min="15" max="15" width="31.21875" customWidth="true"/>
+    <col min="1" max="1" width="14.59765625" customWidth="true"/>
+    <col min="2" max="2" width="13.796875" customWidth="true"/>
+    <col min="3" max="3" width="14.73046875" customWidth="true"/>
+    <col min="4" max="4" width="24.9296875" customWidth="true"/>
+    <col min="5" max="5" width="25.86328125" customWidth="true"/>
+    <col min="6" max="6" width="20.33203125" customWidth="true"/>
+    <col min="7" max="7" width="33.59765625" customWidth="true"/>
+    <col min="8" max="8" width="21.265625" customWidth="true"/>
+    <col min="9" max="9" width="32.86328125" customWidth="true"/>
+    <col min="10" max="10" width="22.33203125" customWidth="true"/>
+    <col min="11" max="11" width="23.265625" customWidth="true"/>
+    <col min="12" max="12" width="17.73046875" customWidth="true"/>
+    <col min="13" max="13" width="31" customWidth="true"/>
+    <col min="14" max="14" width="18.6640625" customWidth="true"/>
+    <col min="15" max="15" width="30.265625" customWidth="true"/>
   </cols>
   <sheetData>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
@@ -1149,7 +1149,7 @@
         <v>-103.60432654936449</v>
       </c>
       <c r="I4" s="0">
-        <v>44.362647030171488</v>
+        <v>44.362647030171487</v>
       </c>
       <c r="J4" s="0">
         <v>0.16011818092593047</v>
@@ -1178,7 +1178,7 @@
         <v>0.23927080437932036</v>
       </c>
       <c r="C5" s="0">
-        <v>129.93522414268981</v>
+        <v>129.9352241426898</v>
       </c>
       <c r="D5" s="0">
         <v>0.24506768956937586</v>
@@ -1227,14 +1227,14 @@
   <dimension ref="A1:H1205"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" customWidth="true"/>
-    <col min="2" max="2" width="6.88671875" customWidth="true"/>
-    <col min="3" max="3" width="6.77734375" customWidth="true"/>
-    <col min="4" max="4" width="15.5546875" customWidth="true"/>
-    <col min="5" max="5" width="20.5546875" customWidth="true"/>
-    <col min="6" max="6" width="18.109375" customWidth="true"/>
-    <col min="7" max="7" width="16.88671875" customWidth="true"/>
-    <col min="8" max="8" width="16.21875" customWidth="true"/>
+    <col min="1" max="1" width="14.59765625" customWidth="true"/>
+    <col min="2" max="2" width="7.06640625" customWidth="true"/>
+    <col min="3" max="3" width="6.86328125" customWidth="true"/>
+    <col min="4" max="4" width="15.796875" customWidth="true"/>
+    <col min="5" max="5" width="20.3984375" customWidth="true"/>
+    <col min="6" max="6" width="17.796875" customWidth="true"/>
+    <col min="7" max="7" width="16.73046875" customWidth="true"/>
+    <col min="8" max="8" width="16.3984375" customWidth="true"/>
   </cols>
   <sheetData>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
@@ -1352,7 +1352,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="0">
-        <v>0.0057858554400725786</v>
+        <v>0.0057858554400725785</v>
       </c>
       <c r="E5" s="0">
         <v>0.0053312317462447549</v>
@@ -1433,7 +1433,7 @@
         <v>0.0052101587627085121</v>
       </c>
       <c r="E8" s="0">
-        <v>0.004855555038354293</v>
+        <v>0.0048555550383542929</v>
       </c>
       <c r="F8" s="0">
         <v>0.0043546277508787054</v>
@@ -1641,7 +1641,7 @@
         <v>0.0039397920568640362</v>
       </c>
       <c r="E16" s="0">
-        <v>0.003784446766010809</v>
+        <v>0.0037844467660108089</v>
       </c>
       <c r="F16" s="0">
         <v>0.0036260164026430033</v>
@@ -1650,7 +1650,7 @@
         <v>0.00015534529085322723</v>
       </c>
       <c r="H16" s="0">
-        <v>0.0003137756542210329</v>
+        <v>0.00031377565422103289</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
@@ -1702,7 +1702,7 @@
         <v>0.00011806439850947778</v>
       </c>
       <c r="H18" s="0">
-        <v>0.00021013996392522895</v>
+        <v>0.00021013996392522894</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
@@ -1855,7 +1855,7 @@
         <v>0.0030193154741144099</v>
       </c>
       <c r="G24" s="0">
-        <v>2.9553465834233472e-05</v>
+        <v>2.9553465834233471e-05</v>
       </c>
       <c r="H24" s="0">
         <v>-4.0143023089169328e-05</v>
@@ -2014,7 +2014,7 @@
         <v>-3.093623528858426e-05</v>
       </c>
       <c r="H30" s="0">
-        <v>-0.00021608089997859513</v>
+        <v>-0.00021608089997859512</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.3">
@@ -2040,7 +2040,7 @@
         <v>-3.8827733109404305e-05</v>
       </c>
       <c r="H31" s="0">
-        <v>-0.00023946598285890138</v>
+        <v>-0.00023946598285890137</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.3">
@@ -2083,7 +2083,7 @@
         <v>0.0021754333356873963</v>
       </c>
       <c r="E33" s="0">
-        <v>0.0022284345293716998</v>
+        <v>0.0022284345293716997</v>
       </c>
       <c r="F33" s="0">
         <v>0.0024572370915491521</v>
@@ -2326,7 +2326,7 @@
         <v>-9.5048504765739544e-05</v>
       </c>
       <c r="H42" s="0">
-        <v>-0.00041126389994375129</v>
+        <v>-0.00041126389994375128</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.3">
@@ -2730,7 +2730,7 @@
         <v>224</v>
       </c>
       <c r="D58" s="0">
-        <v>0.00090832360654587554</v>
+        <v>0.00090832360654587553</v>
       </c>
       <c r="E58" s="0">
         <v>0.0010227297214159847</v>
@@ -2993,7 +2993,7 @@
         <v>0.00064049910922349949</v>
       </c>
       <c r="E68" s="0">
-        <v>0.00074897147260316079</v>
+        <v>0.00074897147260316078</v>
       </c>
       <c r="F68" s="0">
         <v>0.001102913618365349</v>
@@ -3002,7 +3002,7 @@
         <v>-0.0001084723633796613</v>
       </c>
       <c r="H68" s="0">
-        <v>-0.00046241450914184953</v>
+        <v>-0.00046241450914184952</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="69" x14ac:dyDescent="0.3">
@@ -3120,7 +3120,7 @@
         <v>284</v>
       </c>
       <c r="D73" s="0">
-        <v>0.00053784544443359205</v>
+        <v>0.00053784544443359204</v>
       </c>
       <c r="E73" s="0">
         <v>0.00064094014733400459</v>
@@ -3256,13 +3256,13 @@
         <v>0.00054849121427378883</v>
       </c>
       <c r="F78" s="0">
-        <v>0.00087728339622030372</v>
+        <v>0.00087728339622030371</v>
       </c>
       <c r="G78" s="0">
         <v>-9.6846991928702304e-05</v>
       </c>
       <c r="H78" s="0">
-        <v>-0.00042563917387521719</v>
+        <v>-0.00042563917387521718</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="79" x14ac:dyDescent="0.3">
@@ -3308,7 +3308,7 @@
         <v>0.00051535981939042808</v>
       </c>
       <c r="F80" s="0">
-        <v>0.00083803005026462756</v>
+        <v>0.00083803005026462755</v>
       </c>
       <c r="G80" s="0">
         <v>-9.4195040748055309e-05</v>
@@ -3334,7 +3334,7 @@
         <v>0.00049955233719413915</v>
       </c>
       <c r="F81" s="0">
-        <v>0.00081906700814863101</v>
+        <v>0.000819067008148631</v>
       </c>
       <c r="G81" s="0">
         <v>-9.28470319802905e-05</v>
@@ -3360,13 +3360,13 @@
         <v>0.00048422971331234119</v>
       </c>
       <c r="F82" s="0">
-        <v>0.00080053306397032717</v>
+        <v>0.00080053306397032716</v>
       </c>
       <c r="G82" s="0">
         <v>-9.1487457366135809e-05</v>
       </c>
       <c r="H82" s="0">
-        <v>-0.00040779080802412179</v>
+        <v>-0.00040779080802412178</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="83" x14ac:dyDescent="0.3">
@@ -3389,7 +3389,7 @@
         <v>0.0007824185080513318</v>
       </c>
       <c r="G83" s="0">
-        <v>-9.0118488273649954e-05</v>
+        <v>-9.0118488273649953e-05</v>
       </c>
       <c r="H83" s="0">
         <v>-0.00040315992049833488</v>
@@ -3458,10 +3458,10 @@
         <v>336</v>
       </c>
       <c r="D86" s="0">
-        <v>0.00034152209189086008</v>
+        <v>0.00034152209189086007</v>
       </c>
       <c r="E86" s="0">
-        <v>0.00042749712147168183</v>
+        <v>0.00042749712147168182</v>
       </c>
       <c r="F86" s="0">
         <v>0.00073049733902496943</v>
@@ -3490,7 +3490,7 @@
         <v>0.0004143846263132091</v>
       </c>
       <c r="F87" s="0">
-        <v>0.00071396755969166306</v>
+        <v>0.00071396755969166305</v>
       </c>
       <c r="G87" s="0">
         <v>-8.458770676194558e-05</v>
@@ -3574,7 +3574,7 @@
         <v>-8.0429453476648619e-05</v>
       </c>
       <c r="H90" s="0">
-        <v>-0.00036960689025061989</v>
+        <v>-0.00036960689025061988</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="91" x14ac:dyDescent="0.3">
@@ -3782,7 +3782,7 @@
         <v>-6.9586217830304529e-05</v>
       </c>
       <c r="H98" s="0">
-        <v>-0.00033048561104762016</v>
+        <v>-0.00033048561104762015</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="99" x14ac:dyDescent="0.3">
@@ -3796,7 +3796,7 @@
         <v>388</v>
       </c>
       <c r="D99" s="0">
-        <v>0.00021686032754696019</v>
+        <v>0.00021686032754696018</v>
       </c>
       <c r="E99" s="0">
         <v>0.00028513393899062128</v>
@@ -3886,7 +3886,7 @@
         <v>-6.4410421291718161e-05</v>
       </c>
       <c r="H102" s="0">
-        <v>-0.00031121351502829266</v>
+        <v>-0.00031121351502829265</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="103" x14ac:dyDescent="0.3">
@@ -3955,7 +3955,7 @@
         <v>0.00017585181968614796</v>
       </c>
       <c r="E105" s="0">
-        <v>0.00023652200572514543</v>
+        <v>0.00023652200572514542</v>
       </c>
       <c r="F105" s="0">
         <v>0.00047288508711852971</v>
@@ -4224,7 +4224,7 @@
         <v>-4.9210304705710423e-05</v>
       </c>
       <c r="H115" s="0">
-        <v>-0.00025214301689597955</v>
+        <v>-0.00025214301689597954</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="116" x14ac:dyDescent="0.3">
@@ -4247,7 +4247,7 @@
         <v>0.00036763247663308251</v>
       </c>
       <c r="G116" s="0">
-        <v>-4.8154659567957082e-05</v>
+        <v>-4.8154659567957081e-05</v>
       </c>
       <c r="H116" s="0">
         <v>-0.00024788880008248386</v>
@@ -4270,10 +4270,10 @@
         <v>0.00016274843917447529</v>
       </c>
       <c r="F117" s="0">
-        <v>0.00035931364589974558</v>
+        <v>0.00035931364589974557</v>
       </c>
       <c r="G117" s="0">
-        <v>-4.711581510765379e-05</v>
+        <v>-4.7115815107653789e-05</v>
       </c>
       <c r="H117" s="0">
         <v>-0.00024368102183292407</v>
@@ -4328,7 +4328,7 @@
         <v>-4.5088587383124723e-05</v>
       </c>
       <c r="H119" s="0">
-        <v>-0.00023540734667018912</v>
+        <v>-0.00023540734667018911</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="120" x14ac:dyDescent="0.3">
@@ -4351,7 +4351,7 @@
         <v>0.00033546964892081012</v>
       </c>
       <c r="G120" s="0">
-        <v>-4.4100187508468132e-05</v>
+        <v>-4.4100187508468131e-05</v>
       </c>
       <c r="H120" s="0">
         <v>-0.00023134255211087465</v>
@@ -4608,7 +4608,7 @@
         <v>0.00010855068068444907</v>
       </c>
       <c r="F130" s="0">
-        <v>0.00026684043793952982</v>
+        <v>0.00026684043793952981</v>
       </c>
       <c r="G130" s="0">
         <v>-3.5126063871493464e-05</v>
@@ -4628,7 +4628,7 @@
         <v>516</v>
       </c>
       <c r="D131" s="0">
-        <v>7.0903795154437922e-05</v>
+        <v>7.0903795154437921e-05</v>
       </c>
       <c r="E131" s="0">
         <v>0.00010522113715436931</v>
@@ -4637,10 +4637,10 @@
         <v>0.00026080234126113456</v>
       </c>
       <c r="G131" s="0">
-        <v>-3.431734199993139e-05</v>
+        <v>-3.4317341999931389e-05</v>
       </c>
       <c r="H131" s="0">
-        <v>-0.00018989854610669663</v>
+        <v>-0.00018989854610669662</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="132" x14ac:dyDescent="0.3">
@@ -4683,7 +4683,7 @@
         <v>6.6118815903519463e-05</v>
       </c>
       <c r="E133" s="0">
-        <v>9.8865295976943431e-05</v>
+        <v>9.886529597694343e-05</v>
       </c>
       <c r="F133" s="0">
         <v>0.00024913294848374879</v>
@@ -4718,7 +4718,7 @@
         <v>-3.1984011672170511e-05</v>
       </c>
       <c r="H134" s="0">
-        <v>-0.0001796467211810353</v>
+        <v>-0.00017964672118103529</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="135" x14ac:dyDescent="0.3">
@@ -4819,7 +4819,7 @@
         <v>0.00022219300023106108</v>
       </c>
       <c r="G138" s="0">
-        <v>-2.9083144712928279e-05</v>
+        <v>-2.9083144712928278e-05</v>
       </c>
       <c r="H138" s="0">
         <v>-0.00016667113702634244</v>
@@ -5313,7 +5313,7 @@
         <v>0.00014383591925418542</v>
       </c>
       <c r="G157" s="0">
-        <v>-1.8220998105161389e-05</v>
+        <v>-1.8220998105161388e-05</v>
       </c>
       <c r="H157" s="0">
         <v>-0.00011524737137179747</v>
@@ -5385,7 +5385,7 @@
         <v>2.5743967301863141e-05</v>
       </c>
       <c r="E160" s="0">
-        <v>4.263298571160773e-05</v>
+        <v>4.2632985711607729e-05</v>
       </c>
       <c r="F160" s="0">
         <v>0.00013429099029505501</v>
@@ -5931,7 +5931,7 @@
         <v>1.2361157090535315e-05</v>
       </c>
       <c r="E181" s="0">
-        <v>2.2162818347011225e-05</v>
+        <v>2.2162818347011224e-05</v>
       </c>
       <c r="F181" s="0">
         <v>8.304309724430565e-05</v>
@@ -5940,7 +5940,7 @@
         <v>-9.8016612564759094e-06</v>
       </c>
       <c r="H181" s="0">
-        <v>-7.0681940153770329e-05</v>
+        <v>-7.0681940153770328e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="182" x14ac:dyDescent="0.3">
@@ -5986,7 +5986,7 @@
         <v>2.0824082069612095e-05</v>
       </c>
       <c r="F183" s="0">
-        <v>7.9327400082583689e-05</v>
+        <v>7.9327400082583688e-05</v>
       </c>
       <c r="G183" s="0">
         <v>-9.297124052154929e-06</v>
@@ -6067,7 +6067,7 @@
         <v>7.4063246300782448e-05</v>
       </c>
       <c r="G186" s="0">
-        <v>-8.5860452919800228e-06</v>
+        <v>-8.5860452919800227e-06</v>
       </c>
       <c r="H186" s="0">
         <v>-6.3683228696804041e-05</v>
@@ -6318,7 +6318,7 @@
         <v>776</v>
       </c>
       <c r="D196" s="0">
-        <v>7.3194090532938598e-06</v>
+        <v>7.3194090532938597e-06</v>
       </c>
       <c r="E196" s="0">
         <v>1.3889339244979659e-05</v>
@@ -6448,7 +6448,7 @@
         <v>796</v>
       </c>
       <c r="D201" s="0">
-        <v>6.1463173930604094e-06</v>
+        <v>6.1463173930604093e-06</v>
       </c>
       <c r="E201" s="0">
         <v>1.1885946885411006e-05</v>
@@ -6535,7 +6535,7 @@
         <v>4.9054616283059099e-05</v>
       </c>
       <c r="G204" s="0">
-        <v>-5.2906742265655448e-06</v>
+        <v>-5.2906742265655447e-06</v>
       </c>
       <c r="H204" s="0">
         <v>-4.3519861784692349e-05</v>
@@ -6639,7 +6639,7 @@
         <v>4.4763006394691354e-05</v>
       </c>
       <c r="G208" s="0">
-        <v>-4.7441862919319351e-06</v>
+        <v>-4.744186291931935e-06</v>
       </c>
       <c r="H208" s="0">
         <v>-3.9950076525888364e-05</v>
@@ -6922,7 +6922,7 @@
         <v>6.784247818969684e-06</v>
       </c>
       <c r="F219" s="0">
-        <v>3.4799860157776715e-05</v>
+        <v>3.4799860157776714e-05</v>
       </c>
       <c r="G219" s="0">
         <v>-3.5069549339756858e-06</v>
@@ -6980,7 +6980,7 @@
         <v>-3.3183249311463554e-06</v>
       </c>
       <c r="H221" s="0">
-        <v>-3.0186645085579205e-05</v>
+        <v>-3.0186645085579204e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="222" x14ac:dyDescent="0.3">
@@ -7023,13 +7023,13 @@
         <v>2.8498790361266617e-06</v>
       </c>
       <c r="E223" s="0">
-        <v>5.9894020012137062e-06</v>
+        <v>5.9894020012137061e-06</v>
       </c>
       <c r="F223" s="0">
         <v>3.1755347015422233e-05</v>
       </c>
       <c r="G223" s="0">
-        <v>-3.1395229650870445e-06</v>
+        <v>-3.1395229650870444e-06</v>
       </c>
       <c r="H223" s="0">
         <v>-2.8905467979295573e-05</v>
@@ -7098,7 +7098,7 @@
         <v>896</v>
       </c>
       <c r="D226" s="0">
-        <v>2.5663140717093946e-06</v>
+        <v>2.5663140717093945e-06</v>
       </c>
       <c r="E226" s="0">
         <v>5.455000354131549e-06</v>
@@ -7179,7 +7179,7 @@
         <v>2.3109640202851561e-06</v>
       </c>
       <c r="E229" s="0">
-        <v>4.9682804489572241e-06</v>
+        <v>4.968280448957224e-06</v>
       </c>
       <c r="F229" s="0">
         <v>2.7680626115084285e-05</v>
@@ -7205,7 +7205,7 @@
         <v>2.2316237607475393e-06</v>
       </c>
       <c r="E230" s="0">
-        <v>4.8158898244107571e-06</v>
+        <v>4.815889824410757e-06</v>
       </c>
       <c r="F230" s="0">
         <v>2.7054265665776117e-05</v>
@@ -7341,7 +7341,7 @@
         <v>2.4128757331827198e-05</v>
       </c>
       <c r="G235" s="0">
-        <v>-2.2472895528857033e-06</v>
+        <v>-2.2472895528857032e-06</v>
       </c>
       <c r="H235" s="0">
         <v>-2.2254798951365194e-05</v>
@@ -7370,7 +7370,7 @@
         <v>-2.1852166469027248e-06</v>
       </c>
       <c r="H236" s="0">
-        <v>-2.1773147540829594e-05</v>
+        <v>-2.1773147540829593e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="237" x14ac:dyDescent="0.3">
@@ -7422,7 +7422,7 @@
         <v>-2.06603327003813e-06</v>
       </c>
       <c r="H238" s="0">
-        <v>-2.0840078587344339e-05</v>
+        <v>-2.0840078587344338e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="239" x14ac:dyDescent="0.3">
@@ -7474,7 +7474,7 @@
         <v>-1.9531843739966073e-06</v>
       </c>
       <c r="H240" s="0">
-        <v>-1.9945981817161914e-05</v>
+        <v>-1.9945981817161913e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="241" x14ac:dyDescent="0.3">
@@ -7526,7 +7526,7 @@
         <v>-1.8463456846595688e-06</v>
       </c>
       <c r="H242" s="0">
-        <v>-1.9089300874693402e-05</v>
+        <v>-1.9089300874693401e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="243" x14ac:dyDescent="0.3">
@@ -7552,7 +7552,7 @@
         <v>-1.795083129701416e-06</v>
       </c>
       <c r="H243" s="0">
-        <v>-1.8674520607300618e-05</v>
+        <v>-1.8674520607300617e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="244" x14ac:dyDescent="0.3">
@@ -8072,7 +8072,7 @@
         <v>-1.0180732079167433e-06</v>
       </c>
       <c r="H263" s="0">
-        <v>-1.2007308392031966e-05</v>
+        <v>-1.2007308392031965e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="264" x14ac:dyDescent="0.3">
@@ -8095,7 +8095,7 @@
         <v>1.2424254709568516e-05</v>
       </c>
       <c r="G264" s="0">
-        <v>-9.894245270128147e-07</v>
+        <v>-9.8942452701281469e-07</v>
       </c>
       <c r="H264" s="0">
         <v>-1.1743852156128516e-05</v>
@@ -8251,7 +8251,7 @@
         <v>1.0830023340860298e-05</v>
       </c>
       <c r="G270" s="0">
-        <v>-8.3340375356089664e-07</v>
+        <v>-8.3340375356089663e-07</v>
       </c>
       <c r="H270" s="0">
         <v>-1.0278285600283402e-05</v>
@@ -8294,7 +8294,7 @@
         <v>1080</v>
       </c>
       <c r="D272" s="0">
-        <v>5.1450343407949783e-07</v>
+        <v>5.1450343407949782e-07</v>
       </c>
       <c r="E272" s="0">
         <v>1.3014725699739503e-06</v>
@@ -8404,13 +8404,13 @@
         <v>1.1489914023085534e-06</v>
       </c>
       <c r="F276" s="0">
-        <v>9.4403574544595149e-06</v>
+        <v>9.4403574544595148e-06</v>
       </c>
       <c r="G276" s="0">
         <v>-7.0158782800121113e-07</v>
       </c>
       <c r="H276" s="0">
-        <v>-8.9929538801521726e-06</v>
+        <v>-8.9929538801521725e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="277" x14ac:dyDescent="0.3">
@@ -8462,7 +8462,7 @@
         <v>-6.6237671812154164e-07</v>
       </c>
       <c r="H278" s="0">
-        <v>-8.6007458756439316e-06</v>
+        <v>-8.6007458756439315e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="279" x14ac:dyDescent="0.3">
@@ -8667,10 +8667,10 @@
         <v>7.5090820452980072e-06</v>
       </c>
       <c r="G286" s="0">
-        <v>-5.2595214404237978e-07</v>
+        <v>-5.2595214404237977e-07</v>
       </c>
       <c r="H286" s="0">
-        <v>-7.1935980165420186e-06</v>
+        <v>-7.1935980165420185e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="287" x14ac:dyDescent="0.3">
@@ -8904,7 +8904,7 @@
         <v>-4.0533343851326345e-07</v>
       </c>
       <c r="H295" s="0">
-        <v>-5.8808139865686372e-06</v>
+        <v>-5.8808139865686371e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="296" x14ac:dyDescent="0.3">
@@ -8921,7 +8921,7 @@
         <v>2.2246172832704664e-07</v>
       </c>
       <c r="E296" s="0">
-        <v>6.1620550986806552e-07</v>
+        <v>6.1620550986806551e-07</v>
       </c>
       <c r="F296" s="0">
         <v>5.9729002249147549e-06</v>
@@ -8930,7 +8930,7 @@
         <v>-3.9374378154101888e-07</v>
       </c>
       <c r="H296" s="0">
-        <v>-5.7504384965877087e-06</v>
+        <v>-5.7504384965877086e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="297" x14ac:dyDescent="0.3">
@@ -9126,7 +9126,7 @@
         <v>4</v>
       </c>
       <c r="D304" s="0">
-        <v>8.975861193912393e-05</v>
+        <v>8.9758611939123929e-05</v>
       </c>
       <c r="E304" s="0">
         <v>0.0018118767951447478</v>
@@ -9152,7 +9152,7 @@
         <v>8</v>
       </c>
       <c r="D305" s="0">
-        <v>0.00025832278130565501</v>
+        <v>0.000258322781305655</v>
       </c>
       <c r="E305" s="0">
         <v>0.0017769455866225867</v>
@@ -9320,7 +9320,7 @@
         <v>-0.00060238354105391495</v>
       </c>
       <c r="H311" s="0">
-        <v>-0.00067720861179436398</v>
+        <v>-0.00067720861179436397</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="312" x14ac:dyDescent="0.3">
@@ -9580,7 +9580,7 @@
         <v>0.00013754105679995464</v>
       </c>
       <c r="H321" s="0">
-        <v>3.8236985225384435e-06</v>
+        <v>3.8236985225384434e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="322" x14ac:dyDescent="0.3">
@@ -10048,7 +10048,7 @@
         <v>0.00036881591932753542</v>
       </c>
       <c r="H339" s="0">
-        <v>0.00017630158822267567</v>
+        <v>0.00017630158822267566</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="340" x14ac:dyDescent="0.3">
@@ -10169,7 +10169,7 @@
         <v>0.0011708456450633029</v>
       </c>
       <c r="E344" s="0">
-        <v>0.00083166286082627208</v>
+        <v>0.00083166286082627207</v>
       </c>
       <c r="F344" s="0">
         <v>0.0010326058772406818</v>
@@ -10429,7 +10429,7 @@
         <v>0.00093365928733498695</v>
       </c>
       <c r="E354" s="0">
-        <v>0.00068454494700775828</v>
+        <v>0.00068454494700775827</v>
       </c>
       <c r="F354" s="0">
         <v>0.00089492125668050814</v>
@@ -10646,7 +10646,7 @@
         <v>0.00017293470635495903</v>
       </c>
       <c r="H362" s="0">
-        <v>-3.9357412218727858e-05</v>
+        <v>-3.9357412218727857e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="363" x14ac:dyDescent="0.3">
@@ -10660,7 +10660,7 @@
         <v>240</v>
       </c>
       <c r="D363" s="0">
-        <v>0.00073842071793104583</v>
+        <v>0.00073842071793104582</v>
       </c>
       <c r="E363" s="0">
         <v>0.00057452795365952106</v>
@@ -10773,7 +10773,7 @@
         <v>0.00074300224231869602</v>
       </c>
       <c r="G367" s="0">
-        <v>0.00012936684474555477</v>
+        <v>0.00012936684474555476</v>
       </c>
       <c r="H367" s="0">
         <v>-8.2147929672228169e-05</v>
@@ -10972,7 +10972,7 @@
         <v>288</v>
       </c>
       <c r="D375" s="0">
-        <v>0.00052432434626893362</v>
+        <v>0.00052432434626893361</v>
       </c>
       <c r="E375" s="0">
         <v>0.00045483801717059394</v>
@@ -11007,7 +11007,7 @@
         <v>0.00065321377193388718</v>
       </c>
       <c r="G376" s="0">
-        <v>6.2919050946081215e-05</v>
+        <v>6.2919050946081214e-05</v>
       </c>
       <c r="H376" s="0">
         <v>-0.00014422553493429857</v>
@@ -11157,7 +11157,7 @@
         <v>0.00042468095213193567</v>
       </c>
       <c r="E382" s="0">
-        <v>0.00039689444495363667</v>
+        <v>0.00039689444495363666</v>
       </c>
       <c r="F382" s="0">
         <v>0.00059946726312954518</v>
@@ -11709,7 +11709,7 @@
         <v>0.00044386505708519453</v>
       </c>
       <c r="G403" s="0">
-        <v>-4.5090256061115661e-05</v>
+        <v>-4.509025606111566e-05</v>
       </c>
       <c r="H403" s="0">
         <v>-0.00022524336383191463</v>
@@ -11738,7 +11738,7 @@
         <v>-4.6996276483427863e-05</v>
       </c>
       <c r="H404" s="0">
-        <v>-0.000225926789123624</v>
+        <v>-0.00022592678912362399</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="405" x14ac:dyDescent="0.3">
@@ -11862,7 +11862,7 @@
         <v>0.00023464030025652482</v>
       </c>
       <c r="F409" s="0">
-        <v>0.00040734378606553879</v>
+        <v>0.00040734378606553878</v>
       </c>
       <c r="G409" s="0">
         <v>-5.4909954990164543e-05</v>
@@ -11891,7 +11891,7 @@
         <v>0.0004015559993479083</v>
       </c>
       <c r="G410" s="0">
-        <v>-5.6194215807667172e-05</v>
+        <v>-5.6194215807667171e-05</v>
       </c>
       <c r="H410" s="0">
         <v>-0.00022763354988235998</v>
@@ -11940,7 +11940,7 @@
         <v>0.00022132934770380526</v>
       </c>
       <c r="F412" s="0">
-        <v>0.00039022596656431981</v>
+        <v>0.0003902259665643198</v>
       </c>
       <c r="G412" s="0">
         <v>-5.8491441361352637e-05</v>
@@ -11969,7 +11969,7 @@
         <v>0.00038468140017245122</v>
       </c>
       <c r="G413" s="0">
-        <v>-5.9510890929235719e-05</v>
+        <v>-5.9510890929235718e-05</v>
       </c>
       <c r="H413" s="0">
         <v>-0.00022712995626400644</v>
@@ -11998,7 +11998,7 @@
         <v>-6.0448436061824725e-05</v>
       </c>
       <c r="H414" s="0">
-        <v>-0.00022678646459604451</v>
+        <v>-0.0002267864645960445</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="415" x14ac:dyDescent="0.3">
@@ -12122,7 +12122,7 @@
         <v>0.00019313334702166039</v>
       </c>
       <c r="F419" s="0">
-        <v>0.00035302976766013521</v>
+        <v>0.0003530297676601352</v>
       </c>
       <c r="G419" s="0">
         <v>-6.4012249706117989e-05</v>
@@ -12142,7 +12142,7 @@
         <v>468</v>
       </c>
       <c r="D420" s="0">
-        <v>0.00012488978598782533</v>
+        <v>0.00012488978598782532</v>
       </c>
       <c r="E420" s="0">
         <v>0.00018940992540961995</v>
@@ -12359,7 +12359,7 @@
         <v>0.00031036771224077648</v>
       </c>
       <c r="G428" s="0">
-        <v>-6.6557140601157948e-05</v>
+        <v>-6.6557140601157947e-05</v>
       </c>
       <c r="H428" s="0">
         <v>-0.00021483103105157192</v>
@@ -12596,7 +12596,7 @@
         <v>-6.5542985320991184e-05</v>
       </c>
       <c r="H437" s="0">
-        <v>-0.00020236132932746794</v>
+        <v>-0.00020236132932746793</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="438" x14ac:dyDescent="0.3">
@@ -12720,7 +12720,7 @@
         <v>0.00012342495788953233</v>
       </c>
       <c r="F442" s="0">
-        <v>0.00025401938412131535</v>
+        <v>0.00025401938412131534</v>
       </c>
       <c r="G442" s="0">
         <v>-6.3933152828748178e-05</v>
@@ -12795,10 +12795,10 @@
         <v>5.3715297578108527e-05</v>
       </c>
       <c r="E445" s="0">
-        <v>0.0001164231608559757</v>
+        <v>0.00011642316085597569</v>
       </c>
       <c r="F445" s="0">
-        <v>0.0002433447203214854</v>
+        <v>0.00024334472032148539</v>
       </c>
       <c r="G445" s="0">
         <v>-6.2707863277867168e-05</v>
@@ -12853,10 +12853,10 @@
         <v>0.00023647867009827145</v>
       </c>
       <c r="G447" s="0">
-        <v>-6.180334013648322e-05</v>
+        <v>-6.1803340136483219e-05</v>
       </c>
       <c r="H447" s="0">
-        <v>-0.00018630462598370819</v>
+        <v>-0.00018630462598370818</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="448" x14ac:dyDescent="0.3">
@@ -13104,7 +13104,7 @@
         <v>616</v>
       </c>
       <c r="D457" s="0">
-        <v>3.5636609821617631e-05</v>
+        <v>3.563660982161763e-05</v>
       </c>
       <c r="E457" s="0">
         <v>9.2169022062670109e-05</v>
@@ -13133,10 +13133,10 @@
         <v>3.4434833047985739e-05</v>
       </c>
       <c r="E458" s="0">
-        <v>9.0392093665782282e-05</v>
+        <v>9.0392093665782281e-05</v>
       </c>
       <c r="F458" s="0">
-        <v>0.00020203528690997247</v>
+        <v>0.00020203528690997246</v>
       </c>
       <c r="G458" s="0">
         <v>-5.5957260617796542e-05</v>
@@ -13211,7 +13211,7 @@
         <v>3.1064466676519273e-05</v>
       </c>
       <c r="E461" s="0">
-        <v>8.5264224034645669e-05</v>
+        <v>8.5264224034645668e-05</v>
       </c>
       <c r="F461" s="0">
         <v>0.00019354515230498437</v>
@@ -13269,7 +13269,7 @@
         <v>0.00018808421304799123</v>
       </c>
       <c r="G463" s="0">
-        <v>-5.3007468594642462e-05</v>
+        <v>-5.3007468594642461e-05</v>
       </c>
       <c r="H463" s="0">
         <v>-0.00015908338786845916</v>
@@ -13321,10 +13321,10 @@
         <v>0.00018277735596362507</v>
       </c>
       <c r="G465" s="0">
-        <v>-5.1803872850410892e-05</v>
+        <v>-5.1803872850410891e-05</v>
       </c>
       <c r="H465" s="0">
-        <v>-0.00015570453317884697</v>
+        <v>-0.00015570453317884696</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="466" x14ac:dyDescent="0.3">
@@ -13347,7 +13347,7 @@
         <v>0.00018018034481648637</v>
       </c>
       <c r="G466" s="0">
-        <v>-5.1199100778351277e-05</v>
+        <v>-5.1199100778351276e-05</v>
       </c>
       <c r="H466" s="0">
         <v>-0.00015402341533278828</v>
@@ -13624,7 +13624,7 @@
         <v>696</v>
       </c>
       <c r="D477" s="0">
-        <v>1.7899598361920118e-05</v>
+        <v>1.7899598361920117e-05</v>
       </c>
       <c r="E477" s="0">
         <v>6.2444515737068625e-05</v>
@@ -13662,7 +13662,7 @@
         <v>-4.3948865485437577e-05</v>
       </c>
       <c r="H478" s="0">
-        <v>-0.00013445786639513811</v>
+        <v>-0.0001344578663951381</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="479" x14ac:dyDescent="0.3">
@@ -13994,7 +13994,7 @@
         <v>4.7547843836070108e-05</v>
       </c>
       <c r="F491" s="0">
-        <v>0.00012598910528952392</v>
+        <v>0.00012598910528952391</v>
       </c>
       <c r="G491" s="0">
         <v>-3.6520753029548245e-05</v>
@@ -14153,7 +14153,7 @@
         <v>0.00011562270634382026</v>
       </c>
       <c r="G497" s="0">
-        <v>-3.3350271696496198e-05</v>
+        <v>-3.3350271696496197e-05</v>
       </c>
       <c r="H497" s="0">
         <v>-0.00010666681639974183</v>
@@ -14326,7 +14326,7 @@
         <v>804</v>
       </c>
       <c r="D504" s="0">
-        <v>7.0239824278378392e-06</v>
+        <v>7.0239824278378391e-06</v>
       </c>
       <c r="E504" s="0">
         <v>3.6916616264635917e-05</v>
@@ -14404,7 +14404,7 @@
         <v>816</v>
       </c>
       <c r="D507" s="0">
-        <v>6.3288549406006973e-06</v>
+        <v>6.3288549406006972e-06</v>
       </c>
       <c r="E507" s="0">
         <v>3.4822366781625979e-05</v>
@@ -14436,7 +14436,7 @@
         <v>3.4151025684624416e-05</v>
       </c>
       <c r="F508" s="0">
-        <v>9.8782129651582362e-05</v>
+        <v>9.8782129651582361e-05</v>
       </c>
       <c r="G508" s="0">
         <v>-2.8038298534155839e-05</v>
@@ -14621,7 +14621,7 @@
         <v>8.9366252550811371e-05</v>
       </c>
       <c r="G515" s="0">
-        <v>-2.5008003024018006e-05</v>
+        <v>-2.5008003024018005e-05</v>
       </c>
       <c r="H515" s="0">
         <v>-8.4573860990370909e-05</v>
@@ -14716,7 +14716,7 @@
         <v>864</v>
       </c>
       <c r="D519" s="0">
-        <v>4.1698956188229388e-06</v>
+        <v>4.1698956188229387e-06</v>
       </c>
       <c r="E519" s="0">
         <v>2.756791233438958e-05</v>
@@ -15008,7 +15008,7 @@
         <v>2.2253791071896101e-05</v>
       </c>
       <c r="F530" s="0">
-        <v>7.2102262660197895e-05</v>
+        <v>7.2102262660197894e-05</v>
       </c>
       <c r="G530" s="0">
         <v>-1.9410415859742732e-05</v>
@@ -15028,7 +15028,7 @@
         <v>912</v>
       </c>
       <c r="D531" s="0">
-        <v>2.7460558215686192e-06</v>
+        <v>2.7460558215686191e-06</v>
       </c>
       <c r="E531" s="0">
         <v>2.1824759794259528e-05</v>
@@ -15161,7 +15161,7 @@
         <v>2.307114108938265e-06</v>
       </c>
       <c r="E536" s="0">
-        <v>1.9800529450906576e-05</v>
+        <v>1.9800529450906575e-05</v>
       </c>
       <c r="F536" s="0">
         <v>6.6169679696727364e-05</v>
@@ -15213,7 +15213,7 @@
         <v>2.1518195802312791e-06</v>
       </c>
       <c r="E538" s="0">
-        <v>1.9044419326848438e-05</v>
+        <v>1.9044419326848437e-05</v>
       </c>
       <c r="F538" s="0">
         <v>6.4302680719098028e-05</v>
@@ -15271,7 +15271,7 @@
         <v>6.248835972326405e-05</v>
       </c>
       <c r="G540" s="0">
-        <v>-1.6310221645694608e-05</v>
+        <v>-1.6310221645694607e-05</v>
       </c>
       <c r="H540" s="0">
         <v>-6.048139907360178e-05</v>
@@ -15395,7 +15395,7 @@
         <v>1.6859938020050157e-06</v>
       </c>
       <c r="E545" s="0">
-        <v>1.6618277173077299e-05</v>
+        <v>1.6618277173077298e-05</v>
       </c>
       <c r="F545" s="0">
         <v>5.8173372300290877e-05</v>
@@ -15612,7 +15612,7 @@
         <v>-1.2946017397385757e-05</v>
       </c>
       <c r="H553" s="0">
-        <v>-5.0604908439443366e-05</v>
+        <v>-5.0604908439443365e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="554" x14ac:dyDescent="0.3">
@@ -15658,7 +15658,7 @@
         <v>1.3678568807920815e-05</v>
       </c>
       <c r="F555" s="0">
-        <v>5.0416706501259812e-05</v>
+        <v>5.0416706501259811e-05</v>
       </c>
       <c r="G555" s="0">
         <v>-1.2488882460665542e-05</v>
@@ -15918,7 +15918,7 @@
         <v>1.125888337788371e-05</v>
       </c>
       <c r="F565" s="0">
-        <v>4.3694291630768382e-05</v>
+        <v>4.3694291630768381e-05</v>
       </c>
       <c r="G565" s="0">
         <v>-1.0419528216899446e-05</v>
@@ -16097,7 +16097,7 @@
         <v>6.5746820383082287e-07</v>
       </c>
       <c r="E572" s="0">
-        <v>9.8245707270922099e-06</v>
+        <v>9.8245707270922098e-06</v>
       </c>
       <c r="F572" s="0">
         <v>3.9529367454182046e-05</v>
@@ -16227,7 +16227,7 @@
         <v>5.5220067817825767e-07</v>
       </c>
       <c r="E577" s="0">
-        <v>8.9133490520922355e-06</v>
+        <v>8.9133490520922354e-06</v>
       </c>
       <c r="F577" s="0">
         <v>3.6799759505465496e-05</v>
@@ -16262,7 +16262,7 @@
         <v>-8.2082469345991469e-06</v>
       </c>
       <c r="H578" s="0">
-        <v>-3.5743624794979026e-05</v>
+        <v>-3.5743624794979025e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="579" x14ac:dyDescent="0.3">
@@ -16308,13 +16308,13 @@
         <v>8.4077020418023715e-06</v>
       </c>
       <c r="F580" s="0">
-        <v>3.5253322165676369e-05</v>
+        <v>3.5253322165676368e-05</v>
       </c>
       <c r="G580" s="0">
         <v>-7.9103937513163393e-06</v>
       </c>
       <c r="H580" s="0">
-        <v>-3.4756013875190335e-05</v>
+        <v>-3.4756013875190334e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="581" x14ac:dyDescent="0.3">
@@ -16620,10 +16620,10 @@
         <v>6.656147018254263e-06</v>
       </c>
       <c r="F592" s="0">
-        <v>2.9690692514901695e-05</v>
+        <v>2.9690692514901694e-05</v>
       </c>
       <c r="G592" s="0">
-        <v>-6.3290236242583104e-06</v>
+        <v>-6.3290236242583103e-06</v>
       </c>
       <c r="H592" s="0">
         <v>-2.936356912090574e-05</v>
@@ -16640,7 +16640,7 @@
         <v>1160</v>
       </c>
       <c r="D593" s="0">
-        <v>3.1590044805197273e-07</v>
+        <v>3.1590044805197272e-07</v>
       </c>
       <c r="E593" s="0">
         <v>6.5278230284157455e-06</v>
@@ -16692,7 +16692,7 @@
         <v>1168</v>
       </c>
       <c r="D595" s="0">
-        <v>2.9459594242541484e-07</v>
+        <v>2.9459594242541483e-07</v>
       </c>
       <c r="E595" s="0">
         <v>6.2785492354051741e-06</v>
@@ -16851,7 +16851,7 @@
         <v>2.3891898927635176e-07</v>
       </c>
       <c r="E601" s="0">
-        <v>5.5864009257104416e-06</v>
+        <v>5.5864009257104415e-06</v>
       </c>
       <c r="F601" s="0">
         <v>2.6102706215884253e-05</v>
@@ -16860,7 +16860,7 @@
         <v>-5.3474819364340897e-06</v>
       </c>
       <c r="H601" s="0">
-        <v>-2.5863787226607903e-05</v>
+        <v>-2.5863787226607902e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="602" x14ac:dyDescent="0.3">
@@ -16877,7 +16877,7 @@
         <v>2.3072105018301665e-07</v>
       </c>
       <c r="E602" s="0">
-        <v>5.4787005919199226e-06</v>
+        <v>5.4787005919199225e-06</v>
       </c>
       <c r="F602" s="0">
         <v>2.5731823189068673e-05</v>
@@ -17059,7 +17059,7 @@
         <v>0.00082698237710766354</v>
       </c>
       <c r="E609" s="0">
-        <v>0.0022744437176490029</v>
+        <v>0.0022744437176490028</v>
       </c>
       <c r="F609" s="0">
         <v>0.0019713704507875059</v>
@@ -17550,7 +17550,7 @@
         <v>96</v>
       </c>
       <c r="D628" s="0">
-        <v>0.0019760518316770896</v>
+        <v>0.0019760518316770895</v>
       </c>
       <c r="E628" s="0">
         <v>0.0016426467706846647</v>
@@ -17588,7 +17588,7 @@
         <v>0.00036306547857582142</v>
       </c>
       <c r="H629" s="0">
-        <v>0.00045951932873035699</v>
+        <v>0.00045951932873035698</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="630" x14ac:dyDescent="0.3">
@@ -18128,7 +18128,7 @@
         <v>0.001126932104302487</v>
       </c>
       <c r="F650" s="0">
-        <v>0.0011541840277924851</v>
+        <v>0.001154184027792485</v>
       </c>
       <c r="G650" s="0">
         <v>0.00044707352475557459</v>
@@ -18290,7 +18290,7 @@
         <v>0.00038594329963349047</v>
       </c>
       <c r="H656" s="0">
-        <v>0.00033560236672510705</v>
+        <v>0.00033560236672510704</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="657" x14ac:dyDescent="0.3">
@@ -18440,7 +18440,7 @@
         <v>0.00091756335498570005</v>
       </c>
       <c r="F662" s="0">
-        <v>0.00098679803244005921</v>
+        <v>0.0009867980324400592</v>
       </c>
       <c r="G662" s="0">
         <v>0.00031738073417750517</v>
@@ -18466,7 +18466,7 @@
         <v>0.00090198140941210952</v>
       </c>
       <c r="F663" s="0">
-        <v>0.00097399720239253849</v>
+        <v>0.00097399720239253848</v>
       </c>
       <c r="G663" s="0">
         <v>0.00030580298218990036</v>
@@ -18602,7 +18602,7 @@
         <v>0.00024880382370585312</v>
       </c>
       <c r="H668" s="0">
-        <v>0.00016431473990778461</v>
+        <v>0.0001643147399077846</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="669" x14ac:dyDescent="0.3">
@@ -18628,7 +18628,7 @@
         <v>0.00023771360029607952</v>
       </c>
       <c r="H669" s="0">
-        <v>0.00015100060449750521</v>
+        <v>0.0001510006044975052</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="670" x14ac:dyDescent="0.3">
@@ -18677,7 +18677,7 @@
         <v>0.00087739102182120363</v>
       </c>
       <c r="G671" s="0">
-        <v>0.00021596273589108797</v>
+        <v>0.00021596273589108796</v>
       </c>
       <c r="H671" s="0">
         <v>0.00012505553442170351</v>
@@ -18798,7 +18798,7 @@
         <v>288</v>
       </c>
       <c r="D676" s="0">
-        <v>0.00088651299289267455</v>
+        <v>0.00088651299289267454</v>
       </c>
       <c r="E676" s="0">
         <v>0.00072193387677832986</v>
@@ -18810,7 +18810,7 @@
         <v>0.00016457911611434469</v>
       </c>
       <c r="H676" s="0">
-        <v>6.4572533291152061e-05</v>
+        <v>6.457253329115206e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="677" x14ac:dyDescent="0.3">
@@ -18853,7 +18853,7 @@
         <v>0.00084300576439017959</v>
       </c>
       <c r="E678" s="0">
-        <v>0.0006976224902740481</v>
+        <v>0.00069762249027404809</v>
       </c>
       <c r="F678" s="0">
         <v>0.00080075420516850402</v>
@@ -19110,7 +19110,7 @@
         <v>336</v>
       </c>
       <c r="D688" s="0">
-        <v>0.00065007295091012031</v>
+        <v>0.0006500729509101203</v>
       </c>
       <c r="E688" s="0">
         <v>0.00058780832272460766</v>
@@ -19165,7 +19165,7 @@
         <v>0.00061626520615457503</v>
       </c>
       <c r="E690" s="0">
-        <v>0.00056801366315278738</v>
+        <v>0.00056801366315278737</v>
       </c>
       <c r="F690" s="0">
         <v>0.00068462450969773183</v>
@@ -19194,7 +19194,7 @@
         <v>0.00055836772651395939</v>
       </c>
       <c r="F691" s="0">
-        <v>0.00067574350091284628</v>
+        <v>0.00067574350091284627</v>
       </c>
       <c r="G691" s="0">
         <v>4.1565174668296563e-05</v>
@@ -19266,7 +19266,7 @@
         <v>360</v>
       </c>
       <c r="D694" s="0">
-        <v>0.00055316207221769651</v>
+        <v>0.0005531620722176965</v>
       </c>
       <c r="E694" s="0">
         <v>0.00053040167340134153</v>
@@ -19295,10 +19295,10 @@
         <v>0.00053829610906227555</v>
       </c>
       <c r="E695" s="0">
-        <v>0.00052139445884533977</v>
+        <v>0.00052139445884533976</v>
       </c>
       <c r="F695" s="0">
-        <v>0.00064135667012796608</v>
+        <v>0.00064135667012796607</v>
       </c>
       <c r="G695" s="0">
         <v>1.6901650216935788e-05</v>
@@ -19743,7 +19743,7 @@
         <v>0.0005136886895661996</v>
       </c>
       <c r="G712" s="0">
-        <v>-5.488949687247987e-05</v>
+        <v>-5.4889496872479869e-05</v>
       </c>
       <c r="H712" s="0">
         <v>-0.00017889438824600297</v>
@@ -19812,7 +19812,7 @@
         <v>444</v>
       </c>
       <c r="D715" s="0">
-        <v>0.00030729436665533517</v>
+        <v>0.00030729436665533516</v>
       </c>
       <c r="E715" s="0">
         <v>0.00037016634172107538</v>
@@ -19864,7 +19864,7 @@
         <v>452</v>
       </c>
       <c r="D717" s="0">
-        <v>0.00029015256604406797</v>
+        <v>0.00029015256604406796</v>
       </c>
       <c r="E717" s="0">
         <v>0.00035770085520779973</v>
@@ -20026,7 +20026,7 @@
         <v>0.00032276700557742097</v>
       </c>
       <c r="F723" s="0">
-        <v>0.0004449628813527251</v>
+        <v>0.00044496288135272509</v>
       </c>
       <c r="G723" s="0">
         <v>-7.8789094495718956e-05</v>
@@ -20231,7 +20231,7 @@
         <v>0.00019318822714865121</v>
       </c>
       <c r="E731" s="0">
-        <v>0.00028143709502338982</v>
+        <v>0.00028143709502338981</v>
       </c>
       <c r="F731" s="0">
         <v>0.00040082911550831494</v>
@@ -20442,7 +20442,7 @@
         <v>0.00024539942771878366</v>
       </c>
       <c r="F739" s="0">
-        <v>0.00036107276937515749</v>
+        <v>0.00036107276937515748</v>
       </c>
       <c r="G739" s="0">
         <v>-9.2763212296770217e-05</v>
@@ -20861,7 +20861,7 @@
         <v>0.00029299869775181915</v>
       </c>
       <c r="G755" s="0">
-        <v>-9.1778684862769633e-05</v>
+        <v>-9.1778684862769632e-05</v>
       </c>
       <c r="H755" s="0">
         <v>-0.00019820044605016793</v>
@@ -20904,7 +20904,7 @@
         <v>612</v>
       </c>
       <c r="D757" s="0">
-        <v>8.9284331394766563e-05</v>
+        <v>8.9284331394766562e-05</v>
       </c>
       <c r="E757" s="0">
         <v>0.00018029389020310534</v>
@@ -20988,7 +20988,7 @@
         <v>0.00017126380434771433</v>
       </c>
       <c r="F760" s="0">
-        <v>0.00027448136384264729</v>
+        <v>0.00027448136384264728</v>
       </c>
       <c r="G760" s="0">
         <v>-8.9665972247371061e-05</v>
@@ -21095,7 +21095,7 @@
         <v>0.00026051372049970724</v>
       </c>
       <c r="G764" s="0">
-        <v>-8.7571857752047266e-05</v>
+        <v>-8.7571857752047265e-05</v>
       </c>
       <c r="H764" s="0">
         <v>-0.00018816229768328451</v>
@@ -21167,7 +21167,7 @@
         <v>6.6100106309775281e-05</v>
       </c>
       <c r="E767" s="0">
-        <v>0.00015191346419486893</v>
+        <v>0.00015191346419486892</v>
       </c>
       <c r="F767" s="0">
         <v>0.00025050644566793344</v>
@@ -21427,7 +21427,7 @@
         <v>4.8865055712257453e-05</v>
       </c>
       <c r="E777" s="0">
-        <v>0.00012800045846083936</v>
+        <v>0.00012800045846083935</v>
       </c>
       <c r="F777" s="0">
         <v>0.00021984330820873851</v>
@@ -21956,7 +21956,7 @@
         <v>-6.4255544610558637e-05</v>
       </c>
       <c r="H797" s="0">
-        <v>-0.00014269858020652787</v>
+        <v>-0.00014269858020652786</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="798" x14ac:dyDescent="0.3">
@@ -21973,7 +21973,7 @@
         <v>2.5820348125565999e-05</v>
       </c>
       <c r="E798" s="0">
-        <v>8.933128197583388e-05</v>
+        <v>8.9331281975833879e-05</v>
       </c>
       <c r="F798" s="0">
         <v>0.00016712113509207127</v>
@@ -22034,7 +22034,7 @@
         <v>-6.2029243117905851e-05</v>
       </c>
       <c r="H800" s="0">
-        <v>-0.00013851966219131514</v>
+        <v>-0.00013851966219131513</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="801" x14ac:dyDescent="0.3">
@@ -22236,7 +22236,7 @@
         <v>7.5269464154497715e-05</v>
       </c>
       <c r="F808" s="0">
-        <v>0.00014666474194816886</v>
+        <v>0.00014666474194816885</v>
       </c>
       <c r="G808" s="0">
         <v>-5.6236189463643811e-05</v>
@@ -22392,7 +22392,7 @@
         <v>6.7918483288083878e-05</v>
       </c>
       <c r="F814" s="0">
-        <v>0.00013561331427324104</v>
+        <v>0.00013561331427324103</v>
       </c>
       <c r="G814" s="0">
         <v>-5.2072401698238107e-05</v>
@@ -22473,7 +22473,7 @@
         <v>0.00013040391607272838</v>
       </c>
       <c r="G817" s="0">
-        <v>-5.0059159845020863e-05</v>
+        <v>-5.0059159845020862e-05</v>
       </c>
       <c r="H817" s="0">
         <v>-0.00011594631486533529</v>
@@ -22545,7 +22545,7 @@
         <v>1.3190231464402213e-05</v>
       </c>
       <c r="E820" s="0">
-        <v>6.1285415327061067e-05</v>
+        <v>6.1285415327061066e-05</v>
       </c>
       <c r="F820" s="0">
         <v>0.00012539462971047392</v>
@@ -22918,7 +22918,7 @@
         <v>-3.9626784866779441e-05</v>
       </c>
       <c r="H834" s="0">
-        <v>-9.5853561870971454e-05</v>
+        <v>-9.5853561870971453e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="835" x14ac:dyDescent="0.3">
@@ -23120,10 +23120,10 @@
         <v>4.2044646049369661e-05</v>
       </c>
       <c r="F842" s="0">
-        <v>9.4086323381924287e-05</v>
+        <v>9.4086323381924286e-05</v>
       </c>
       <c r="G842" s="0">
-        <v>-3.5320920213243002e-05</v>
+        <v>-3.5320920213243001e-05</v>
       </c>
       <c r="H842" s="0">
         <v>-8.7362597545797627e-05</v>
@@ -23192,7 +23192,7 @@
         <v>964</v>
       </c>
       <c r="D845" s="0">
-        <v>6.1327299831942626e-06</v>
+        <v>6.1327299831942625e-06</v>
       </c>
       <c r="E845" s="0">
         <v>3.9938824475728808e-05</v>
@@ -23400,7 +23400,7 @@
         <v>996</v>
       </c>
       <c r="D853" s="0">
-        <v>4.7979762452244881e-06</v>
+        <v>4.797976245224488e-06</v>
       </c>
       <c r="E853" s="0">
         <v>3.4824708055241457e-05</v>
@@ -23487,7 +23487,7 @@
         <v>7.8367967244050767e-05</v>
       </c>
       <c r="G856" s="0">
-        <v>-2.8704582231618355e-05</v>
+        <v>-2.8704582231618354e-05</v>
       </c>
       <c r="H856" s="0">
         <v>-7.3992049742038009e-05</v>
@@ -23510,7 +23510,7 @@
         <v>3.2518730844762783e-05</v>
       </c>
       <c r="F857" s="0">
-        <v>7.7351371145475043e-05</v>
+        <v>7.7351371145475042e-05</v>
       </c>
       <c r="G857" s="0">
         <v>-2.8275098555375212e-05</v>
@@ -23530,7 +23530,7 @@
         <v>1016</v>
       </c>
       <c r="D858" s="0">
-        <v>4.1153382211109951e-06</v>
+        <v>4.115338221110995e-06</v>
       </c>
       <c r="E858" s="0">
         <v>3.1966501844561233e-05</v>
@@ -23828,7 +23828,7 @@
         <v>-2.3541560568012084e-05</v>
       </c>
       <c r="H869" s="0">
-        <v>-6.3197828210636952e-05</v>
+        <v>-6.3197828210636951e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="870" x14ac:dyDescent="0.3">
@@ -23871,7 +23871,7 @@
         <v>2.7606980016215108e-06</v>
       </c>
       <c r="E871" s="0">
-        <v>2.5585561257551008e-05</v>
+        <v>2.5585561257551007e-05</v>
       </c>
       <c r="F871" s="0">
         <v>6.4428808591064575e-05</v>
@@ -24368,7 +24368,7 @@
         <v>1.8478381878498822e-05</v>
       </c>
       <c r="F890" s="0">
-        <v>5.0273527304289329e-05</v>
+        <v>5.0273527304289328e-05</v>
       </c>
       <c r="G890" s="0">
         <v>-1.6938709507704036e-05</v>
@@ -24475,7 +24475,7 @@
         <v>4.7715238139781887e-05</v>
       </c>
       <c r="G894" s="0">
-        <v>-1.5893296808450026e-05</v>
+        <v>-1.5893296808450025e-05</v>
       </c>
       <c r="H894" s="0">
         <v>-4.6353730520281943e-05</v>
@@ -24573,7 +24573,7 @@
         <v>1.2039430614949828e-06</v>
       </c>
       <c r="E898" s="0">
-        <v>1.6112248237126992e-05</v>
+        <v>1.6112248237126991e-05</v>
       </c>
       <c r="F898" s="0">
         <v>4.5287133662925714e-05</v>
@@ -24628,7 +24628,7 @@
         <v>1.556966240351331e-05</v>
       </c>
       <c r="F900" s="0">
-        <v>4.4119817070687384e-05</v>
+        <v>4.4119817070687383e-05</v>
       </c>
       <c r="G900" s="0">
         <v>-1.4437531011223331e-05</v>
@@ -24651,7 +24651,7 @@
         <v>1.0978469210311638e-06</v>
       </c>
       <c r="E901" s="0">
-        <v>1.5305260353396015e-05</v>
+        <v>1.5305260353396014e-05</v>
       </c>
       <c r="F901" s="0">
         <v>4.3547490959889349e-05</v>
@@ -24813,7 +24813,7 @@
         <v>0.0072088976261778202</v>
       </c>
       <c r="G907" s="0">
-        <v>0.00051081252626420781</v>
+        <v>0.0005108125262642078</v>
       </c>
       <c r="H907" s="0">
         <v>-0.0001751691922718384</v>
@@ -25012,7 +25012,7 @@
         <v>40</v>
       </c>
       <c r="D915" s="0">
-        <v>0.0054983077653212587</v>
+        <v>0.0054983077653212586</v>
       </c>
       <c r="E915" s="0">
         <v>0.0052244253029515393</v>
@@ -25073,7 +25073,7 @@
         <v>0.0053453991646137703</v>
       </c>
       <c r="G917" s="0">
-        <v>0.00022759449448832726</v>
+        <v>0.00022759449448832725</v>
       </c>
       <c r="H917" s="0">
         <v>-0.00017540672630095983</v>
@@ -25142,7 +25142,7 @@
         <v>60</v>
       </c>
       <c r="D920" s="0">
-        <v>0.0047139090747363392</v>
+        <v>0.0047139090747363391</v>
       </c>
       <c r="E920" s="0">
         <v>0.0045476443107084919</v>
@@ -25232,7 +25232,7 @@
         <v>0.0001136402116262954</v>
       </c>
       <c r="H923" s="0">
-        <v>-0.00016925823823581068</v>
+        <v>-0.00016925823823581067</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="924" x14ac:dyDescent="0.3">
@@ -25327,7 +25327,7 @@
         <v>0.0038000929469164269</v>
       </c>
       <c r="E927" s="0">
-        <v>0.0037448432236422418</v>
+        <v>0.0037448432236422417</v>
       </c>
       <c r="F927" s="0">
         <v>0.0039636146482778193</v>
@@ -25379,10 +25379,10 @@
         <v>0.0035731815385739614</v>
       </c>
       <c r="E929" s="0">
-        <v>0.0035426873531942522</v>
+        <v>0.0035426873531942521</v>
       </c>
       <c r="F929" s="0">
-        <v>0.0037334787297266981</v>
+        <v>0.003733478729726698</v>
       </c>
       <c r="G929" s="0">
         <v>3.0494185379709247e-05</v>
@@ -25405,7 +25405,7 @@
         <v>0.0034648585739821256</v>
       </c>
       <c r="E930" s="0">
-        <v>0.0034457393301911494</v>
+        <v>0.0034457393301911493</v>
       </c>
       <c r="F930" s="0">
         <v>0.0036234711660786405</v>
@@ -25532,7 +25532,7 @@
         <v>120</v>
       </c>
       <c r="D935" s="0">
-        <v>0.0029705554821044178</v>
+        <v>0.0029705554821044177</v>
       </c>
       <c r="E935" s="0">
         <v>0.002999372362023342</v>
@@ -25567,7 +25567,7 @@
         <v>0.0030282489808903944</v>
       </c>
       <c r="G936" s="0">
-        <v>-3.6791061278142277e-05</v>
+        <v>-3.6791061278142276e-05</v>
       </c>
       <c r="H936" s="0">
         <v>-0.00014774752286293409</v>
@@ -25596,7 +25596,7 @@
         <v>-4.4281375463295185e-05</v>
       </c>
       <c r="H937" s="0">
-        <v>-0.00014584365631488319</v>
+        <v>-0.00014584365631488318</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="938" x14ac:dyDescent="0.3">
@@ -25668,7 +25668,7 @@
         <v>0.0026108285346037544</v>
       </c>
       <c r="F940" s="0">
-        <v>0.0026868046612042547</v>
+        <v>0.0026868046612042546</v>
       </c>
       <c r="G940" s="0">
         <v>-6.4057956860072256e-05</v>
@@ -25714,7 +25714,7 @@
         <v>148</v>
       </c>
       <c r="D942" s="0">
-        <v>0.0023946976398988591</v>
+        <v>0.002394697639898859</v>
       </c>
       <c r="E942" s="0">
         <v>0.002469889573081638</v>
@@ -25899,7 +25899,7 @@
         <v>0.0019304728765660499</v>
       </c>
       <c r="E949" s="0">
-        <v>0.0020338770138903888</v>
+        <v>0.0020338770138903887</v>
       </c>
       <c r="F949" s="0">
         <v>0.0020527508850232334</v>
@@ -25954,7 +25954,7 @@
         <v>0.001924083317980397</v>
       </c>
       <c r="F951" s="0">
-        <v>0.0019335637913216013</v>
+        <v>0.0019335637913216012</v>
       </c>
       <c r="G951" s="0">
         <v>-0.00010888296903606843</v>
@@ -26055,7 +26055,7 @@
         <v>0.0016048937689367457</v>
       </c>
       <c r="E955" s="0">
-        <v>0.0017219567788608363</v>
+        <v>0.0017219567788608362</v>
       </c>
       <c r="F955" s="0">
         <v>0.0017155485695007598</v>
@@ -26419,7 +26419,7 @@
         <v>0.001042971225202433</v>
       </c>
       <c r="E969" s="0">
-        <v>0.0011676603931481231</v>
+        <v>0.001167660393148123</v>
       </c>
       <c r="F969" s="0">
         <v>0.0011286487753131326</v>
@@ -26480,7 +26480,7 @@
         <v>-0.00012393394964668172</v>
       </c>
       <c r="H971" s="0">
-        <v>-8.2423764159323581e-05</v>
+        <v>-8.242376415932358e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="972" x14ac:dyDescent="0.3">
@@ -26766,7 +26766,7 @@
         <v>-0.00011508395737034715</v>
       </c>
       <c r="H982" s="0">
-        <v>-6.6088948488830617e-05</v>
+        <v>-6.6088948488830616e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="983" x14ac:dyDescent="0.3">
@@ -26884,7 +26884,7 @@
         <v>328</v>
       </c>
       <c r="D987" s="0">
-        <v>0.00059926661937504192</v>
+        <v>0.00059926661937504191</v>
       </c>
       <c r="E987" s="0">
         <v>0.00070861317749895962</v>
@@ -26974,7 +26974,7 @@
         <v>-0.00010561475727675343</v>
       </c>
       <c r="H990" s="0">
-        <v>-5.5870905515852804e-05</v>
+        <v>-5.5870905515852803e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="991" x14ac:dyDescent="0.3">
@@ -27072,13 +27072,13 @@
         <v>0.00058352084609870382</v>
       </c>
       <c r="F994" s="0">
-        <v>0.00053436379184787671</v>
+        <v>0.0005343637918478767</v>
       </c>
       <c r="G994" s="0">
         <v>-0.00010042522047149085</v>
       </c>
       <c r="H994" s="0">
-        <v>-5.1268166220663737e-05</v>
+        <v>-5.1268166220663736e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="995" x14ac:dyDescent="0.3">
@@ -27303,7 +27303,7 @@
         <v>0.00036619042571446836</v>
       </c>
       <c r="E1003" s="0">
-        <v>0.00045457203346605316</v>
+        <v>0.00045457203346605315</v>
       </c>
       <c r="F1003" s="0">
         <v>0.0004082603259101279</v>
@@ -27456,7 +27456,7 @@
         <v>416</v>
       </c>
       <c r="D1009" s="0">
-        <v>0.00030443148909651961</v>
+        <v>0.0003044314890965196</v>
       </c>
       <c r="E1009" s="0">
         <v>0.00038485778105637702</v>
@@ -27641,7 +27641,7 @@
         <v>0.00024541583984618036</v>
       </c>
       <c r="E1016" s="0">
-        <v>0.0003169183768530985</v>
+        <v>0.00031691837685309849</v>
       </c>
       <c r="F1016" s="0">
         <v>0.00027674631465919797</v>
@@ -27670,7 +27670,7 @@
         <v>0.00030824569224220352</v>
       </c>
       <c r="F1017" s="0">
-        <v>0.00026859193906792048</v>
+        <v>0.00026859193906792047</v>
       </c>
       <c r="G1017" s="0">
         <v>-7.0269768628362971e-05</v>
@@ -27771,13 +27771,13 @@
         <v>0.00021040436510875372</v>
       </c>
       <c r="E1021" s="0">
-        <v>0.00027586422809811046</v>
+        <v>0.00027586422809811045</v>
       </c>
       <c r="F1021" s="0">
         <v>0.00023830737776303664</v>
       </c>
       <c r="G1021" s="0">
-        <v>-6.5459862989356732e-05</v>
+        <v>-6.5459862989356731e-05</v>
       </c>
       <c r="H1021" s="0">
         <v>-2.7903012654282916e-05</v>
@@ -28031,7 +28031,7 @@
         <v>0.00015465325208698623</v>
       </c>
       <c r="E1031" s="0">
-        <v>0.00020902167267395443</v>
+        <v>0.00020902167267395442</v>
       </c>
       <c r="F1031" s="0">
         <v>0.00017670497267017411</v>
@@ -28066,7 +28066,7 @@
         <v>-5.3336800320345957e-05</v>
       </c>
       <c r="H1032" s="0">
-        <v>-2.1533477995695853e-05</v>
+        <v>-2.1533477995695852e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1033" x14ac:dyDescent="0.3">
@@ -28092,7 +28092,7 @@
         <v>-5.2319580835521768e-05</v>
       </c>
       <c r="H1033" s="0">
-        <v>-2.1026518562145805e-05</v>
+        <v>-2.1026518562145804e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1034" x14ac:dyDescent="0.3">
@@ -28210,7 +28210,7 @@
         <v>532</v>
       </c>
       <c r="D1038" s="0">
-        <v>0.0001246729037738845</v>
+        <v>0.00012467290377388449</v>
       </c>
       <c r="E1038" s="0">
         <v>0.00017212282690276572</v>
@@ -28268,7 +28268,7 @@
         <v>0.00016283121232279541</v>
       </c>
       <c r="F1040" s="0">
-        <v>0.00013500471183272627</v>
+        <v>0.00013500471183272626</v>
       </c>
       <c r="G1040" s="0">
         <v>-4.5602785453201464e-05</v>
@@ -28317,7 +28317,7 @@
         <v>0.00011022847507622107</v>
       </c>
       <c r="E1042" s="0">
-        <v>0.00015404118200713357</v>
+        <v>0.00015404118200713356</v>
       </c>
       <c r="F1042" s="0">
         <v>0.000127166050377619</v>
@@ -28352,7 +28352,7 @@
         <v>-4.293890322209491e-05</v>
       </c>
       <c r="H1043" s="0">
-        <v>-1.6532243630273776e-05</v>
+        <v>-1.6532243630273775e-05</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1044" x14ac:dyDescent="0.3">
@@ -28733,7 +28733,7 @@
         <v>6.7356683834839907e-05</v>
       </c>
       <c r="E1058" s="0">
-        <v>9.8816696564466505e-05</v>
+        <v>9.8816696564466504e-05</v>
       </c>
       <c r="F1058" s="0">
         <v>7.8804176699730815e-05</v>
@@ -28840,7 +28840,7 @@
         <v>8.8435921107835855e-05</v>
       </c>
       <c r="F1062" s="0">
-        <v>6.9918765139630356e-05</v>
+        <v>6.9918765139630355e-05</v>
       </c>
       <c r="G1062" s="0">
         <v>-2.8883088691488406e-05</v>
@@ -28895,7 +28895,7 @@
         <v>6.5859132539786079e-05</v>
       </c>
       <c r="G1064" s="0">
-        <v>-2.7665122400765014e-05</v>
+        <v>-2.7665122400765013e-05</v>
       </c>
       <c r="H1064" s="0">
         <v>-9.8623229005503072e-06</v>
@@ -28912,7 +28912,7 @@
         <v>640</v>
       </c>
       <c r="D1065" s="0">
-        <v>5.4299235541103742e-05</v>
+        <v>5.4299235541103741e-05</v>
       </c>
       <c r="E1065" s="0">
         <v>8.1372466980493099e-05</v>
@@ -28941,7 +28941,7 @@
         <v>5.2653124335897486e-05</v>
       </c>
       <c r="E1066" s="0">
-        <v>7.9145654672731583e-05</v>
+        <v>7.9145654672731582e-05</v>
       </c>
       <c r="F1066" s="0">
         <v>6.2035210865511004e-05</v>
@@ -29028,7 +29028,7 @@
         <v>-2.4816020360642969e-05</v>
       </c>
       <c r="H1069" s="0">
-        <v>-8.7033651763528895e-06</v>
+        <v>-8.7033651763528894e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1070" x14ac:dyDescent="0.3">
@@ -29051,7 +29051,7 @@
         <v>5.5040551409097143e-05</v>
       </c>
       <c r="G1070" s="0">
-        <v>-2.4278531579495226e-05</v>
+        <v>-2.4278531579495225e-05</v>
       </c>
       <c r="H1070" s="0">
         <v>-8.4877446013648412e-06</v>
@@ -29097,7 +29097,7 @@
         <v>4.3773042443387261e-05</v>
       </c>
       <c r="E1072" s="0">
-        <v>6.7007688100276551e-05</v>
+        <v>6.700768810027655e-05</v>
       </c>
       <c r="F1072" s="0">
         <v>5.1844779624976685e-05</v>
@@ -29204,13 +29204,13 @@
         <v>5.9968475211965508e-05</v>
       </c>
       <c r="F1076" s="0">
-        <v>4.599912240853372e-05</v>
+        <v>4.5999122408533719e-05</v>
       </c>
       <c r="G1076" s="0">
         <v>-2.1266916397451171e-05</v>
       </c>
       <c r="H1076" s="0">
-        <v>-7.2975635940193828e-06</v>
+        <v>-7.2975635940193827e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1077" x14ac:dyDescent="0.3">
@@ -29227,7 +29227,7 @@
         <v>3.752829976236258e-05</v>
       </c>
       <c r="E1077" s="0">
-        <v>5.8327397539935371e-05</v>
+        <v>5.832739753993537e-05</v>
       </c>
       <c r="F1077" s="0">
         <v>4.4643750715688431e-05</v>
@@ -29250,7 +29250,7 @@
         <v>692</v>
       </c>
       <c r="D1078" s="0">
-        <v>3.6390608703997664e-05</v>
+        <v>3.6390608703997663e-05</v>
       </c>
       <c r="E1078" s="0">
         <v>5.6731229062546528e-05</v>
@@ -29363,7 +29363,7 @@
         <v>3.8442915417550636e-05</v>
       </c>
       <c r="G1082" s="0">
-        <v>-1.8597123121144477e-05</v>
+        <v>-1.8597123121144476e-05</v>
       </c>
       <c r="H1082" s="0">
         <v>-6.2684718687562626e-06</v>
@@ -29392,7 +29392,7 @@
         <v>-1.8183111000341397e-05</v>
       </c>
       <c r="H1083" s="0">
-        <v>-6.1111310164357067e-06</v>
+        <v>-6.1111310164357066e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1084" x14ac:dyDescent="0.3">
@@ -29519,7 +29519,7 @@
         <v>3.2127955239571727e-05</v>
       </c>
       <c r="G1088" s="0">
-        <v>-1.6236975286271667e-05</v>
+        <v>-1.6236975286271666e-05</v>
       </c>
       <c r="H1088" s="0">
         <v>-5.3798125449595396e-06</v>
@@ -29721,7 +29721,7 @@
         <v>2.0909183808797744e-05</v>
       </c>
       <c r="E1096" s="0">
-        <v>3.4428243627454084e-05</v>
+        <v>3.4428243627454083e-05</v>
       </c>
       <c r="F1096" s="0">
         <v>2.5291355882807408e-05</v>
@@ -29730,7 +29730,7 @@
         <v>-1.3519059818656339e-05</v>
       </c>
       <c r="H1096" s="0">
-        <v>-4.3821720740096633e-06</v>
+        <v>-4.3821720740096632e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1097" x14ac:dyDescent="0.3">
@@ -30016,7 +30016,7 @@
         <v>-1.0469396791526173e-05</v>
       </c>
       <c r="H1107" s="0">
-        <v>-3.298034066936656e-06</v>
+        <v>-3.2980340669366559e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1108" x14ac:dyDescent="0.3">
@@ -30068,7 +30068,7 @@
         <v>-9.98962083449535e-06</v>
       </c>
       <c r="H1109" s="0">
-        <v>-3.1311320594598245e-06</v>
+        <v>-3.1311320594598244e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1110" x14ac:dyDescent="0.3">
@@ -30085,7 +30085,7 @@
         <v>1.3588237101507604e-05</v>
       </c>
       <c r="E1110" s="0">
-        <v>2.3345822022331546e-05</v>
+        <v>2.3345822022331545e-05</v>
       </c>
       <c r="F1110" s="0">
         <v>1.6639026344468956e-05</v>
@@ -30143,7 +30143,7 @@
         <v>1.5672928993596444e-05</v>
       </c>
       <c r="G1112" s="0">
-        <v>-9.3087016243209098e-06</v>
+        <v>-9.3087016243209097e-06</v>
       </c>
       <c r="H1112" s="0">
         <v>-2.8960736295003907e-06</v>
@@ -30169,7 +30169,7 @@
         <v>1.5211123567979153e-05</v>
       </c>
       <c r="G1113" s="0">
-        <v>-9.0916528989872853e-06</v>
+        <v>-9.0916528989872852e-06</v>
       </c>
       <c r="H1113" s="0">
         <v>-2.8216056050923165e-06</v>
@@ -30215,7 +30215,7 @@
         <v>1.1649714224158772e-05</v>
       </c>
       <c r="E1115" s="0">
-        <v>2.0321564295060201e-05</v>
+        <v>2.03215642950602e-05</v>
       </c>
       <c r="F1115" s="0">
         <v>1.4327933297191222e-05</v>
@@ -30241,7 +30241,7 @@
         <v>1.1296546726849867e-05</v>
       </c>
       <c r="E1116" s="0">
-        <v>1.9765451015416666e-05</v>
+        <v>1.9765451015416665e-05</v>
       </c>
       <c r="F1116" s="0">
         <v>1.3905758390558965e-05</v>
@@ -30293,7 +30293,7 @@
         <v>1.062200656085841e-05</v>
       </c>
       <c r="E1118" s="0">
-        <v>1.8698463236170614e-05</v>
+        <v>1.8698463236170613e-05</v>
       </c>
       <c r="F1118" s="0">
         <v>1.3098360405552594e-05</v>
@@ -30458,7 +30458,7 @@
         <v>-7.0002438391467491e-06</v>
       </c>
       <c r="H1124" s="0">
-        <v>-2.1161339162952687e-06</v>
+        <v>-2.1161339162952686e-06</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1125" x14ac:dyDescent="0.3">
@@ -30533,7 +30533,7 @@
         <v>1.0007303955919154e-05</v>
       </c>
       <c r="G1127" s="0">
-        <v>-6.5148330550813271e-06</v>
+        <v>-6.514833055081327e-06</v>
       </c>
       <c r="H1127" s="0">
         <v>-1.9557363197755467e-06</v>
@@ -30608,7 +30608,7 @@
         <v>1.3402969567377627e-05</v>
       </c>
       <c r="F1130" s="0">
-        <v>9.148512292993257e-06</v>
+        <v>9.1485122929932569e-06</v>
       </c>
       <c r="G1130" s="0">
         <v>-6.0616904071595721e-06</v>
@@ -30735,13 +30735,13 @@
         <v>6.2939587834262807e-06</v>
       </c>
       <c r="E1135" s="0">
-        <v>1.1666725958403333e-05</v>
+        <v>1.1666725958403332e-05</v>
       </c>
       <c r="F1135" s="0">
         <v>7.877821165065583e-06</v>
       </c>
       <c r="G1135" s="0">
-        <v>-5.3727671749770519e-06</v>
+        <v>-5.3727671749770518e-06</v>
       </c>
       <c r="H1135" s="0">
         <v>-1.5838623816393024e-06</v>
@@ -30972,7 +30972,7 @@
         <v>9.0885653499095686e-06</v>
       </c>
       <c r="F1144" s="0">
-        <v>6.0187495585909208e-06</v>
+        <v>6.0187495585909207e-06</v>
       </c>
       <c r="G1144" s="0">
         <v>-4.3176932408114298e-06</v>
@@ -30995,7 +30995,7 @@
         <v>4.6262404957958204e-06</v>
       </c>
       <c r="E1145" s="0">
-        <v>8.8398506441611836e-06</v>
+        <v>8.8398506441611835e-06</v>
       </c>
       <c r="F1145" s="0">
         <v>5.8414061148271807e-06</v>
@@ -31151,7 +31151,7 @@
         <v>3.8460133967344673e-06</v>
       </c>
       <c r="E1151" s="0">
-        <v>7.4841500429342216e-06</v>
+        <v>7.4841500429342215e-06</v>
       </c>
       <c r="F1151" s="0">
         <v>4.8818470751999406e-06</v>
@@ -31177,7 +31177,7 @@
         <v>3.7294193842286102e-06</v>
       </c>
       <c r="E1152" s="0">
-        <v>7.2793412415403172e-06</v>
+        <v>7.2793412415403171e-06</v>
       </c>
       <c r="F1152" s="0">
         <v>4.7380026497398138e-06</v>
@@ -31238,7 +31238,7 @@
         <v>-3.3796564130096437e-06</v>
       </c>
       <c r="H1154" s="0">
-        <v>-9.5617607204195341e-07</v>
+        <v>-9.561760720419534e-07</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1155" x14ac:dyDescent="0.3">
@@ -31287,7 +31287,7 @@
         <v>4.2037783829703533e-06</v>
       </c>
       <c r="G1156" s="0">
-        <v>-3.2173063843410392e-06</v>
+        <v>-3.2173063843410391e-06</v>
       </c>
       <c r="H1156" s="0">
         <v>-9.0644432561337221e-07</v>
@@ -31440,7 +31440,7 @@
         <v>5.5155396289007977e-06</v>
       </c>
       <c r="F1162" s="0">
-        <v>3.5132299998113913e-06</v>
+        <v>3.5132299998113912e-06</v>
       </c>
       <c r="G1162" s="0">
         <v>-2.7743092562843307e-06</v>
@@ -31466,10 +31466,10 @@
         <v>5.3646031760029518e-06</v>
       </c>
       <c r="F1163" s="0">
-        <v>3.4097121011456587e-06</v>
+        <v>3.4097121011456586e-06</v>
       </c>
       <c r="G1163" s="0">
-        <v>-2.7064747105763181e-06</v>
+        <v>-2.706474710576318e-06</v>
       </c>
       <c r="H1163" s="0">
         <v>-7.5158363571902484e-07</v>
@@ -31674,7 +31674,7 @@
         <v>4.2966932227609516e-06</v>
       </c>
       <c r="F1171" s="0">
-        <v>2.6841497245916672e-06</v>
+        <v>2.6841497245916671e-06</v>
       </c>
       <c r="G1171" s="0">
         <v>-2.2188182351193546e-06</v>
@@ -31732,7 +31732,7 @@
         <v>-2.1109463535822355e-06</v>
       </c>
       <c r="H1173" s="0">
-        <v>-5.7450149271595045e-07</v>
+        <v>-5.7450149271595044e-07</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1174" x14ac:dyDescent="0.3">
@@ -31862,7 +31862,7 @@
         <v>-1.8631248654033019e-06</v>
       </c>
       <c r="H1178" s="0">
-        <v>-5.0206340582794586e-07</v>
+        <v>-5.0206340582794585e-07</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1179" x14ac:dyDescent="0.3">
@@ -32330,7 +32330,7 @@
         <v>-1.1847538109432161e-06</v>
       </c>
       <c r="H1196" s="0">
-        <v>-3.0836817810246522e-07</v>
+        <v>-3.0836817810246521e-07</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1197" x14ac:dyDescent="0.3">
@@ -32577,16 +32577,16 @@
   <dimension ref="A1:J5"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" customWidth="true"/>
-    <col min="2" max="2" width="15.5546875" customWidth="true"/>
-    <col min="3" max="3" width="23.77734375" customWidth="true"/>
-    <col min="4" max="4" width="21.33203125" customWidth="true"/>
-    <col min="5" max="5" width="20.44140625" customWidth="true"/>
-    <col min="6" max="6" width="18" customWidth="true"/>
-    <col min="7" max="7" width="20.5546875" customWidth="true"/>
-    <col min="8" max="8" width="18.109375" customWidth="true"/>
-    <col min="9" max="9" width="23.44140625" customWidth="true"/>
-    <col min="10" max="10" width="21" customWidth="true"/>
+    <col min="1" max="1" width="14.59765625" customWidth="true"/>
+    <col min="2" max="2" width="15.796875" customWidth="true"/>
+    <col min="3" max="3" width="23.53125" customWidth="true"/>
+    <col min="4" max="4" width="20.9296875" customWidth="true"/>
+    <col min="5" max="5" width="20.19921875" customWidth="true"/>
+    <col min="6" max="6" width="17.59765625" customWidth="true"/>
+    <col min="7" max="7" width="20.33203125" customWidth="true"/>
+    <col min="8" max="8" width="17.73046875" customWidth="true"/>
+    <col min="9" max="9" width="23.06640625" customWidth="true"/>
+    <col min="10" max="10" width="20.46484375" customWidth="true"/>
   </cols>
   <sheetData>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
@@ -32650,7 +32650,7 @@
         <v>0.067708789109633863</v>
       </c>
       <c r="J2" s="0">
-        <v>0.21588336835553818</v>
+        <v>0.21588336835553817</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
@@ -32658,7 +32658,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="0">
-        <v>8.975861193912393e-05</v>
+        <v>8.9758611939123929e-05</v>
       </c>
       <c r="C3" s="0">
         <v>0.0018118767951447478</v>
@@ -32673,7 +32673,7 @@
         <v>0.0017405893821060045</v>
       </c>
       <c r="G3" s="0">
-        <v>0.00022996073794544697</v>
+        <v>0.00022996073794544696</v>
       </c>
       <c r="H3" s="0">
         <v>0.00024515901472358769</v>

</xml_diff>